<commit_message>
Add 101 Audius links verified by track names and duration; refresh catalog and Excel
</commit_message>
<xml_diff>
--- a/Ch-D_music_catalog_updated.xlsx
+++ b/Ch-D_music_catalog_updated.xlsx
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="C6" s="3" t="n">
-        <v>1</v>
+        <v>102</v>
       </c>
     </row>
     <row r="7">
@@ -1292,7 +1292,11 @@
       <c r="H16" s="9" t="inlineStr"/>
       <c r="I16" s="10" t="inlineStr"/>
       <c r="J16" s="9" t="inlineStr"/>
-      <c r="K16" s="9" t="inlineStr"/>
+      <c r="K16" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/cript-cover-den-1</t>
+        </is>
+      </c>
       <c r="L16" s="11" t="n">
         <v>0.002778356481481481</v>
       </c>
@@ -1328,7 +1332,11 @@
       <c r="H17" s="9" t="inlineStr"/>
       <c r="I17" s="10" t="inlineStr"/>
       <c r="J17" s="9" t="inlineStr"/>
-      <c r="K17" s="9" t="inlineStr"/>
+      <c r="K17" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/cryptonit-–-проклятие-крипты</t>
+        </is>
+      </c>
       <c r="L17" s="11" t="n">
         <v>0.002508101851851852</v>
       </c>
@@ -1364,7 +1372,11 @@
       <c r="H18" s="9" t="inlineStr"/>
       <c r="I18" s="10" t="inlineStr"/>
       <c r="J18" s="9" t="inlineStr"/>
-      <c r="K18" s="9" t="inlineStr"/>
+      <c r="K18" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/digital-fury</t>
+        </is>
+      </c>
       <c r="L18" s="11" t="n">
         <v>0.002633217592592592</v>
       </c>
@@ -1408,7 +1420,11 @@
       <c r="H19" s="9" t="inlineStr"/>
       <c r="I19" s="10" t="inlineStr"/>
       <c r="J19" s="9" t="inlineStr"/>
-      <c r="K19" s="9" t="inlineStr"/>
+      <c r="K19" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/dominus-agonetti-rivendare</t>
+        </is>
+      </c>
       <c r="L19" s="11" t="n">
         <v>0.003843055555555556</v>
       </c>
@@ -1452,7 +1468,11 @@
       <c r="H20" s="9" t="inlineStr"/>
       <c r="I20" s="10" t="inlineStr"/>
       <c r="J20" s="9" t="inlineStr"/>
-      <c r="K20" s="9" t="inlineStr"/>
+      <c r="K20" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/dominus-agonetti-—-opera-sessions_-part-i-praeludium-in-ruinis-stratholmi-baro-tenebrosus</t>
+        </is>
+      </c>
       <c r="L20" s="11" t="n">
         <v>0.003261921296296296</v>
       </c>
@@ -1496,7 +1516,11 @@
       <c r="H21" s="9" t="inlineStr"/>
       <c r="I21" s="10" t="inlineStr"/>
       <c r="J21" s="9" t="inlineStr"/>
-      <c r="K21" s="9" t="inlineStr"/>
+      <c r="K21" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/dominus-agonetti-—-opera-sessions_-part-ii-duetus-in-ruinis-stratholmi-aria-rivendari-et-isidis</t>
+        </is>
+      </c>
       <c r="L21" s="11" t="n">
         <v>0.003152777777777777</v>
       </c>
@@ -1536,7 +1560,11 @@
       <c r="H22" s="9" t="inlineStr"/>
       <c r="I22" s="10" t="inlineStr"/>
       <c r="J22" s="9" t="inlineStr"/>
-      <c r="K22" s="9" t="inlineStr"/>
+      <c r="K22" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/edovuaruhaindo-fujōnaru-te-no-kayō</t>
+        </is>
+      </c>
       <c r="L22" s="11" t="n">
         <v>0.002778356481481481</v>
       </c>
@@ -1580,7 +1608,11 @@
       <c r="H23" s="9" t="inlineStr"/>
       <c r="I23" s="10" t="inlineStr"/>
       <c r="J23" s="9" t="inlineStr"/>
-      <c r="K23" s="9" t="inlineStr"/>
+      <c r="K23" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/fakmod-sirus</t>
+        </is>
+      </c>
       <c r="L23" s="11" t="n">
         <v>0.001800810185185185</v>
       </c>
@@ -1620,7 +1652,11 @@
       <c r="H24" s="9" t="inlineStr"/>
       <c r="I24" s="10" t="inlineStr"/>
       <c r="J24" s="9" t="inlineStr"/>
-      <c r="K24" s="9" t="inlineStr"/>
+      <c r="K24" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/fordring-о-король</t>
+        </is>
+      </c>
       <c r="L24" s="11" t="n">
         <v>0.001606134259259259</v>
       </c>
@@ -1664,7 +1700,11 @@
       <c r="H25" s="9" t="inlineStr"/>
       <c r="I25" s="10" t="inlineStr"/>
       <c r="J25" s="9" t="inlineStr"/>
-      <c r="K25" s="9" t="inlineStr"/>
+      <c r="K25" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/fuckmode-wow-sirus</t>
+        </is>
+      </c>
       <c r="L25" s="11" t="n">
         <v>0.001800578703703704</v>
       </c>
@@ -1708,7 +1748,11 @@
       <c r="H26" s="9" t="inlineStr"/>
       <c r="I26" s="10" t="inlineStr"/>
       <c r="J26" s="9" t="inlineStr"/>
-      <c r="K26" s="9" t="inlineStr"/>
+      <c r="K26" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/greywick-hill-мэрри-хоуп</t>
+        </is>
+      </c>
       <c r="L26" s="11" t="n">
         <v>0.00335150462962963</v>
       </c>
@@ -1748,7 +1792,11 @@
       <c r="H27" s="9" t="inlineStr"/>
       <c r="I27" s="10" t="inlineStr"/>
       <c r="J27" s="9" t="inlineStr"/>
-      <c r="K27" s="9" t="inlineStr"/>
+      <c r="K27" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/hastwood-владыка-черного-алмаза</t>
+        </is>
+      </c>
       <c r="L27" s="11" t="n">
         <v>0.002384953703703704</v>
       </c>
@@ -1788,7 +1836,11 @@
       <c r="H28" s="9" t="inlineStr"/>
       <c r="I28" s="10" t="inlineStr"/>
       <c r="J28" s="9" t="inlineStr"/>
-      <c r="K28" s="9" t="inlineStr"/>
+      <c r="K28" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/hastwood-ужас-в-вандермаре</t>
+        </is>
+      </c>
       <c r="L28" s="11" t="n">
         <v>0.002778356481481481</v>
       </c>
@@ -1824,7 +1876,11 @@
       <c r="H29" s="9" t="inlineStr"/>
       <c r="I29" s="10" t="inlineStr"/>
       <c r="J29" s="9" t="inlineStr"/>
-      <c r="K29" s="9" t="inlineStr"/>
+      <c r="K29" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/heilung_-_traust_skysoundcc</t>
+        </is>
+      </c>
       <c r="L29" s="11" t="n">
         <v>0.006855324074074074</v>
       </c>
@@ -1864,7 +1920,11 @@
       <c r="H30" s="9" t="inlineStr"/>
       <c r="I30" s="10" t="inlineStr"/>
       <c r="J30" s="9" t="inlineStr"/>
-      <c r="K30" s="9" t="inlineStr"/>
+      <c r="K30" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/hestia-discordiam-sugere</t>
+        </is>
+      </c>
       <c r="L30" s="11" t="n">
         <v>0.001683912037037037</v>
       </c>
@@ -1908,7 +1968,11 @@
       <c r="H31" s="9" t="inlineStr"/>
       <c r="I31" s="10" t="inlineStr"/>
       <c r="J31" s="9" t="inlineStr"/>
-      <c r="K31" s="9" t="inlineStr"/>
+      <c r="K31" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/homabrut-три-ночи</t>
+        </is>
+      </c>
       <c r="L31" s="11" t="n">
         <v>0.003156134259259259</v>
       </c>
@@ -1952,7 +2016,11 @@
       <c r="H32" s="9" t="inlineStr"/>
       <c r="I32" s="10" t="inlineStr"/>
       <c r="J32" s="9" t="inlineStr"/>
-      <c r="K32" s="9" t="inlineStr"/>
+      <c r="K32" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/kanye-brown-прогрелись-в-котле</t>
+        </is>
+      </c>
       <c r="L32" s="11" t="n">
         <v>0.003093055555555555</v>
       </c>
@@ -1992,7 +2060,11 @@
       <c r="H33" s="9" t="inlineStr"/>
       <c r="I33" s="10" t="inlineStr"/>
       <c r="J33" s="9" t="inlineStr"/>
-      <c r="K33" s="9" t="inlineStr"/>
+      <c r="K33" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/kushnerit-cursed-crypt</t>
+        </is>
+      </c>
       <c r="L33" s="11" t="n">
         <v>0.002783564814814815</v>
       </c>
@@ -2032,7 +2104,11 @@
       <c r="H34" s="9" t="inlineStr"/>
       <c r="I34" s="10" t="inlineStr"/>
       <c r="J34" s="9" t="inlineStr"/>
-      <c r="K34" s="9" t="inlineStr"/>
+      <c r="K34" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/lightfair-мор-ладим</t>
+        </is>
+      </c>
       <c r="L34" s="11" t="n">
         <v>0.002145023148148149</v>
       </c>
@@ -2076,7 +2152,11 @@
       <c r="H35" s="9" t="inlineStr"/>
       <c r="I35" s="10" t="inlineStr"/>
       <c r="J35" s="9" t="inlineStr"/>
-      <c r="K35" s="9" t="inlineStr"/>
+      <c r="K35" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/morgenshtern-x-chd-саркофаг</t>
+        </is>
+      </c>
       <c r="L35" s="11" t="n">
         <v>0.002070023148148148</v>
       </c>
@@ -2116,7 +2196,11 @@
       <c r="H36" s="9" t="inlineStr"/>
       <c r="I36" s="10" t="inlineStr"/>
       <c r="J36" s="9" t="inlineStr"/>
-      <c r="K36" s="9" t="inlineStr"/>
+      <c r="K36" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/mrcrow-блю-юр</t>
+        </is>
+      </c>
       <c r="L36" s="11" t="n">
         <v>0.002141898148148148</v>
       </c>
@@ -2168,7 +2252,11 @@
       <c r="H37" s="9" t="inlineStr"/>
       <c r="I37" s="10" t="inlineStr"/>
       <c r="J37" s="9" t="inlineStr"/>
-      <c r="K37" s="9" t="inlineStr"/>
+      <c r="K37" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/nagvar-жизнь-хороша</t>
+        </is>
+      </c>
       <c r="L37" s="11" t="n">
         <v>0.002015277777777778</v>
       </c>
@@ -2212,7 +2300,11 @@
       <c r="H38" s="9" t="inlineStr"/>
       <c r="I38" s="10" t="inlineStr"/>
       <c r="J38" s="9" t="inlineStr"/>
-      <c r="K38" s="9" t="inlineStr"/>
+      <c r="K38" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/nasramka-за-калич-да</t>
+        </is>
+      </c>
       <c r="L38" s="11" t="n">
         <v>0.001210532407407407</v>
       </c>
@@ -2248,7 +2340,11 @@
       <c r="H39" s="9" t="inlineStr"/>
       <c r="I39" s="10" t="inlineStr"/>
       <c r="J39" s="9" t="inlineStr"/>
-      <c r="K39" s="9" t="inlineStr"/>
+      <c r="K39" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/neizvesten_-_podo_mnoj_penis_bolshoj_ochen_full_skysoundcc</t>
+        </is>
+      </c>
       <c r="L39" s="11" t="n">
         <v>0.001571064814814815</v>
       </c>
@@ -2288,7 +2384,11 @@
       <c r="H40" s="9" t="inlineStr"/>
       <c r="I40" s="10" t="inlineStr"/>
       <c r="J40" s="9" t="inlineStr"/>
-      <c r="K40" s="9" t="inlineStr"/>
+      <c r="K40" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/neoromant-о-король</t>
+        </is>
+      </c>
       <c r="L40" s="11" t="n">
         <v>0.001606134259259259</v>
       </c>
@@ -2328,7 +2428,11 @@
       <c r="H41" s="9" t="inlineStr"/>
       <c r="I41" s="10" t="inlineStr"/>
       <c r="J41" s="9" t="inlineStr"/>
-      <c r="K41" s="9" t="inlineStr"/>
+      <c r="K41" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/neuromant-singularity</t>
+        </is>
+      </c>
       <c r="L41" s="11" t="n">
         <v>0.002292476851851852</v>
       </c>
@@ -2368,7 +2472,11 @@
       <c r="H42" s="9" t="inlineStr"/>
       <c r="I42" s="10" t="inlineStr"/>
       <c r="J42" s="9" t="inlineStr"/>
-      <c r="K42" s="9" t="inlineStr"/>
+      <c r="K42" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/neuromant-agonito-no-kokoro</t>
+        </is>
+      </c>
       <c r="L42" s="11" t="n">
         <v>0.00226724537037037</v>
       </c>
@@ -2408,7 +2516,11 @@
       <c r="H43" s="9" t="inlineStr"/>
       <c r="I43" s="10" t="inlineStr"/>
       <c r="J43" s="9" t="inlineStr"/>
-      <c r="K43" s="9" t="inlineStr"/>
+      <c r="K43" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/neuromant-crypt</t>
+        </is>
+      </c>
       <c r="L43" s="11" t="n">
         <v>0.002778356481481481</v>
       </c>
@@ -2448,7 +2560,11 @@
       <c r="H44" s="9" t="inlineStr"/>
       <c r="I44" s="10" t="inlineStr"/>
       <c r="J44" s="9" t="inlineStr"/>
-      <c r="K44" s="9" t="inlineStr"/>
+      <c r="K44" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/neuromant-destiny</t>
+        </is>
+      </c>
       <c r="L44" s="11" t="n">
         <v>0.001761342592592593</v>
       </c>
@@ -2492,7 +2608,11 @@
       <c r="H45" s="9" t="inlineStr"/>
       <c r="I45" s="10" t="inlineStr"/>
       <c r="J45" s="9" t="inlineStr"/>
-      <c r="K45" s="9" t="inlineStr"/>
+      <c r="K45" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/neuromant-for-that-is-our-curse-arseny-kotofeev</t>
+        </is>
+      </c>
       <c r="L45" s="11" t="n">
         <v>0.002830324074074074</v>
       </c>
@@ -2532,7 +2652,11 @@
       <c r="H46" s="9" t="inlineStr"/>
       <c r="I46" s="10" t="inlineStr"/>
       <c r="J46" s="9" t="inlineStr"/>
-      <c r="K46" s="9" t="inlineStr"/>
+      <c r="K46" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/neuromant-mikurunomicon</t>
+        </is>
+      </c>
       <c r="L46" s="11" t="n">
         <v>0.001929398148148148</v>
       </c>
@@ -2576,7 +2700,11 @@
       <c r="H47" s="9" t="inlineStr"/>
       <c r="I47" s="10" t="inlineStr"/>
       <c r="J47" s="9" t="inlineStr"/>
-      <c r="K47" s="9" t="inlineStr"/>
+      <c r="K47" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/neuromant-singularity-1</t>
+        </is>
+      </c>
       <c r="L47" s="11" t="n">
         <v>0.002051157407407407</v>
       </c>
@@ -2616,7 +2744,11 @@
       <c r="H48" s="9" t="inlineStr"/>
       <c r="I48" s="10" t="inlineStr"/>
       <c r="J48" s="9" t="inlineStr"/>
-      <c r="K48" s="9" t="inlineStr"/>
+      <c r="K48" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/neuromant-артас-сын-мой-v-20</t>
+        </is>
+      </c>
       <c r="L48" s="11" t="n">
         <v>0.001666898148148148</v>
       </c>
@@ -2656,7 +2788,11 @@
       <c r="H49" s="9" t="inlineStr"/>
       <c r="I49" s="10" t="inlineStr"/>
       <c r="J49" s="9" t="inlineStr"/>
-      <c r="K49" s="9" t="inlineStr"/>
+      <c r="K49" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/neuromant-артас-сын-мой</t>
+        </is>
+      </c>
       <c r="L49" s="11" t="n">
         <v>0.001621990740740741</v>
       </c>
@@ -2696,7 +2832,11 @@
       <c r="H50" s="9" t="inlineStr"/>
       <c r="I50" s="10" t="inlineStr"/>
       <c r="J50" s="9" t="inlineStr"/>
-      <c r="K50" s="9" t="inlineStr"/>
+      <c r="K50" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/neuromant-баллада-об-андратосе</t>
+        </is>
+      </c>
       <c r="L50" s="11" t="n">
         <v>0.002778356481481481</v>
       </c>
@@ -2736,7 +2876,11 @@
       <c r="H51" s="9" t="inlineStr"/>
       <c r="I51" s="10" t="inlineStr"/>
       <c r="J51" s="9" t="inlineStr"/>
-      <c r="K51" s="9" t="inlineStr"/>
+      <c r="K51" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/neuromant-в-кругу-семьи-акт-iv</t>
+        </is>
+      </c>
       <c r="L51" s="11" t="n">
         <v>0.002709953703703704</v>
       </c>
@@ -2776,7 +2920,11 @@
       <c r="H52" s="9" t="inlineStr"/>
       <c r="I52" s="10" t="inlineStr"/>
       <c r="J52" s="9" t="inlineStr"/>
-      <c r="K52" s="9" t="inlineStr"/>
+      <c r="K52" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/neuromant-владыка-черной-длани-opening</t>
+        </is>
+      </c>
       <c r="L52" s="11" t="n">
         <v>0.002068634259259259</v>
       </c>
@@ -2816,7 +2964,11 @@
       <c r="H53" s="9" t="inlineStr"/>
       <c r="I53" s="10" t="inlineStr"/>
       <c r="J53" s="9" t="inlineStr"/>
-      <c r="K53" s="9" t="inlineStr"/>
+      <c r="K53" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/neuromant-воспоминание-о-лоретте</t>
+        </is>
+      </c>
       <c r="L53" s="11" t="n">
         <v>0.002171064814814815</v>
       </c>
@@ -2856,7 +3008,11 @@
       <c r="H54" s="9" t="inlineStr"/>
       <c r="I54" s="10" t="inlineStr"/>
       <c r="J54" s="9" t="inlineStr"/>
-      <c r="K54" s="9" t="inlineStr"/>
+      <c r="K54" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/neuromant-день-кузнечного-камня</t>
+        </is>
+      </c>
       <c r="L54" s="11" t="n">
         <v>0.001871990740740741</v>
       </c>
@@ -2896,7 +3052,11 @@
       <c r="H55" s="9" t="inlineStr"/>
       <c r="I55" s="10" t="inlineStr"/>
       <c r="J55" s="9" t="inlineStr"/>
-      <c r="K55" s="9" t="inlineStr"/>
+      <c r="K55" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/neuromant-дерьмадемон</t>
+        </is>
+      </c>
       <c r="L55" s="11" t="n">
         <v>0.002778356481481481</v>
       </c>
@@ -2936,7 +3096,11 @@
       <c r="H56" s="9" t="inlineStr"/>
       <c r="I56" s="10" t="inlineStr"/>
       <c r="J56" s="9" t="inlineStr"/>
-      <c r="K56" s="9" t="inlineStr"/>
+      <c r="K56" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/neuromant-клеть-nu-metal</t>
+        </is>
+      </c>
       <c r="L56" s="11" t="n">
         <v>0.001781134259259259</v>
       </c>
@@ -2976,7 +3140,11 @@
       <c r="H57" s="9" t="inlineStr"/>
       <c r="I57" s="10" t="inlineStr"/>
       <c r="J57" s="9" t="inlineStr"/>
-      <c r="K57" s="9" t="inlineStr"/>
+      <c r="K57" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/neuromant-клеть</t>
+        </is>
+      </c>
       <c r="L57" s="11" t="n">
         <v>0.002253935185185185</v>
       </c>
@@ -3016,7 +3184,11 @@
       <c r="H58" s="9" t="inlineStr"/>
       <c r="I58" s="10" t="inlineStr"/>
       <c r="J58" s="9" t="inlineStr"/>
-      <c r="K58" s="9" t="inlineStr"/>
+      <c r="K58" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/neuromant-край-бесконечно-истерзанный</t>
+        </is>
+      </c>
       <c r="L58" s="11" t="n">
         <v>0.001496412037037037</v>
       </c>
@@ -3056,7 +3228,11 @@
       <c r="H59" s="9" t="inlineStr"/>
       <c r="I59" s="10" t="inlineStr"/>
       <c r="J59" s="9" t="inlineStr"/>
-      <c r="K59" s="9" t="inlineStr"/>
+      <c r="K59" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/neuromant-миша-пошли-exclusive-lovesong-fm-radio-mix-r</t>
+        </is>
+      </c>
       <c r="L59" s="11" t="n">
         <v>0.001665046296296296</v>
       </c>
@@ -3096,7 +3272,11 @@
       <c r="H60" s="9" t="inlineStr"/>
       <c r="I60" s="10" t="inlineStr"/>
       <c r="J60" s="9" t="inlineStr"/>
-      <c r="K60" s="9" t="inlineStr"/>
+      <c r="K60" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/neuromant-ненависть</t>
+        </is>
+      </c>
       <c r="L60" s="11" t="n">
         <v>0.001736689814814815</v>
       </c>
@@ -3140,7 +3320,11 @@
       <c r="H61" s="9" t="inlineStr"/>
       <c r="I61" s="10" t="inlineStr"/>
       <c r="J61" s="9" t="inlineStr"/>
-      <c r="K61" s="9" t="inlineStr"/>
+      <c r="K61" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/neuromant-поднимите-веки-выше</t>
+        </is>
+      </c>
       <c r="L61" s="11" t="n">
         <v>0.002789699074074074</v>
       </c>
@@ -3180,7 +3364,11 @@
       <c r="H62" s="9" t="inlineStr"/>
       <c r="I62" s="10" t="inlineStr"/>
       <c r="J62" s="9" t="inlineStr"/>
-      <c r="K62" s="9" t="inlineStr"/>
+      <c r="K62" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/neuromant-полый</t>
+        </is>
+      </c>
       <c r="L62" s="11" t="n">
         <v>0.002554398148148148</v>
       </c>
@@ -3220,7 +3408,11 @@
       <c r="H63" s="9" t="inlineStr"/>
       <c r="I63" s="10" t="inlineStr"/>
       <c r="J63" s="9" t="inlineStr"/>
-      <c r="K63" s="9" t="inlineStr"/>
+      <c r="K63" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/neuromant-последний-полет-бабочки</t>
+        </is>
+      </c>
       <c r="L63" s="11" t="n">
         <v>0.001967824074074074</v>
       </c>
@@ -3260,7 +3452,11 @@
       <c r="H64" s="9" t="inlineStr"/>
       <c r="I64" s="10" t="inlineStr"/>
       <c r="J64" s="9" t="inlineStr"/>
-      <c r="K64" s="9" t="inlineStr"/>
+      <c r="K64" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/neuromant-проклятье-крипты-darkwave</t>
+        </is>
+      </c>
       <c r="L64" s="11" t="n">
         <v>0.002778356481481481</v>
       </c>
@@ -3300,7 +3496,11 @@
       <c r="H65" s="9" t="inlineStr"/>
       <c r="I65" s="10" t="inlineStr"/>
       <c r="J65" s="9" t="inlineStr"/>
-      <c r="K65" s="9" t="inlineStr"/>
+      <c r="K65" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/neuromant-проклятье-крипты</t>
+        </is>
+      </c>
       <c r="L65" s="11" t="n">
         <v>0.002783564814814815</v>
       </c>
@@ -3344,7 +3544,11 @@
       <c r="H66" s="9" t="inlineStr"/>
       <c r="I66" s="10" t="inlineStr"/>
       <c r="J66" s="9" t="inlineStr"/>
-      <c r="K66" s="9" t="inlineStr"/>
+      <c r="K66" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/neuromant-роксолана</t>
+        </is>
+      </c>
       <c r="L66" s="11" t="n">
         <v>0.002012268518518519</v>
       </c>
@@ -3384,7 +3588,11 @@
       <c r="H67" s="9" t="inlineStr"/>
       <c r="I67" s="10" t="inlineStr"/>
       <c r="J67" s="9" t="inlineStr"/>
-      <c r="K67" s="9" t="inlineStr"/>
+      <c r="K67" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/neuromant-слияние-вечности</t>
+        </is>
+      </c>
       <c r="L67" s="11" t="n">
         <v>0.001932523148148148</v>
       </c>
@@ -3424,7 +3632,11 @@
       <c r="H68" s="9" t="inlineStr"/>
       <c r="I68" s="10" t="inlineStr"/>
       <c r="J68" s="9" t="inlineStr"/>
-      <c r="K68" s="9" t="inlineStr"/>
+      <c r="K68" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/neuromant-терон</t>
+        </is>
+      </c>
       <c r="L68" s="11" t="n">
         <v>0.002457523148148148</v>
       </c>
@@ -3464,7 +3676,11 @@
       <c r="H69" s="9" t="inlineStr"/>
       <c r="I69" s="10" t="inlineStr"/>
       <c r="J69" s="9" t="inlineStr"/>
-      <c r="K69" s="9" t="inlineStr"/>
+      <c r="K69" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/neuromant-эйдолон-1</t>
+        </is>
+      </c>
       <c r="L69" s="11" t="n">
         <v>0.002783564814814815</v>
       </c>
@@ -3504,7 +3720,11 @@
       <c r="H70" s="9" t="inlineStr"/>
       <c r="I70" s="10" t="inlineStr"/>
       <c r="J70" s="9" t="inlineStr"/>
-      <c r="K70" s="9" t="inlineStr"/>
+      <c r="K70" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/neuromant-эйдолон-2</t>
+        </is>
+      </c>
       <c r="L70" s="11" t="n">
         <v>0.002783564814814815</v>
       </c>
@@ -3544,7 +3764,11 @@
       <c r="H71" s="9" t="inlineStr"/>
       <c r="I71" s="10" t="inlineStr"/>
       <c r="J71" s="9" t="inlineStr"/>
-      <c r="K71" s="9" t="inlineStr"/>
+      <c r="K71" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/neuromant-эйдолон</t>
+        </is>
+      </c>
       <c r="L71" s="11" t="n">
         <v>0.003102199074074074</v>
       </c>
@@ -3584,7 +3808,11 @@
       <c r="H72" s="9" t="inlineStr"/>
       <c r="I72" s="10" t="inlineStr"/>
       <c r="J72" s="9" t="inlineStr"/>
-      <c r="K72" s="9" t="inlineStr"/>
+      <c r="K72" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/neuromant-я-был-первым</t>
+        </is>
+      </c>
       <c r="L72" s="11" t="n">
         <v>0.002488657407407407</v>
       </c>
@@ -3624,7 +3852,11 @@
       <c r="H73" s="9" t="inlineStr"/>
       <c r="I73" s="10" t="inlineStr"/>
       <c r="J73" s="9" t="inlineStr"/>
-      <c r="K73" s="9" t="inlineStr"/>
+      <c r="K73" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/neuromanta-singilarityvol2</t>
+        </is>
+      </c>
       <c r="L73" s="11" t="n">
         <v>0.002250810185185185</v>
       </c>
@@ -3664,7 +3896,11 @@
       <c r="H74" s="9" t="inlineStr"/>
       <c r="I74" s="10" t="inlineStr"/>
       <c r="J74" s="9" t="inlineStr"/>
-      <c r="K74" s="9" t="inlineStr"/>
+      <c r="K74" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/nuromanta-antipod-v-0666</t>
+        </is>
+      </c>
       <c r="L74" s="11" t="n">
         <v>0.002544212962962963</v>
       </c>
@@ -3700,7 +3936,11 @@
       <c r="H75" s="9" t="inlineStr"/>
       <c r="I75" s="10" t="inlineStr"/>
       <c r="J75" s="9" t="inlineStr"/>
-      <c r="K75" s="9" t="inlineStr"/>
+      <c r="K75" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/orchestra-de-la-poh-bain-russe</t>
+        </is>
+      </c>
       <c r="L75" s="11" t="n">
         <v>0.001703935185185185</v>
       </c>
@@ -3736,7 +3976,11 @@
       <c r="H76" s="9" t="inlineStr"/>
       <c r="I76" s="10" t="inlineStr"/>
       <c r="J76" s="9" t="inlineStr"/>
-      <c r="K76" s="9" t="inlineStr"/>
+      <c r="K76" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/powerwolf_ai_-_govnovoz_skysoundcc</t>
+        </is>
+      </c>
       <c r="L76" s="11" t="n">
         <v>0.002279398148148148</v>
       </c>
@@ -3772,7 +4016,11 @@
       <c r="H77" s="9" t="inlineStr"/>
       <c r="I77" s="10" t="inlineStr"/>
       <c r="J77" s="9" t="inlineStr"/>
-      <c r="K77" s="9" t="inlineStr"/>
+      <c r="K77" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/samhain-ball</t>
+        </is>
+      </c>
       <c r="L77" s="11" t="n">
         <v>0.001583564814814815</v>
       </c>
@@ -3812,7 +4060,11 @@
       <c r="H78" s="9" t="inlineStr"/>
       <c r="I78" s="10" t="inlineStr"/>
       <c r="J78" s="9" t="inlineStr"/>
-      <c r="K78" s="9" t="inlineStr"/>
+      <c r="K78" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/shizzard-entertaiment-skyborne</t>
+        </is>
+      </c>
       <c r="L78" s="11" t="n">
         <v>0.002309953703703704</v>
       </c>
@@ -3856,7 +4108,11 @@
       <c r="H79" s="9" t="inlineStr"/>
       <c r="I79" s="10" t="inlineStr"/>
       <c r="J79" s="9" t="inlineStr"/>
-      <c r="K79" s="9" t="inlineStr"/>
+      <c r="K79" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/sleep-my-turtling</t>
+        </is>
+      </c>
       <c r="L79" s="11" t="n">
         <v>0.004698611111111111</v>
       </c>
@@ -3900,7 +4156,11 @@
       <c r="H80" s="9" t="inlineStr"/>
       <c r="I80" s="10" t="inlineStr"/>
       <c r="J80" s="9" t="inlineStr"/>
-      <c r="K80" s="9" t="inlineStr"/>
+      <c r="K80" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/teron-я-был-первым-remastered</t>
+        </is>
+      </c>
       <c r="L80" s="11" t="n">
         <v>0.002138310185185185</v>
       </c>
@@ -3940,7 +4200,11 @@
       <c r="H81" s="9" t="inlineStr"/>
       <c r="I81" s="10" t="inlineStr"/>
       <c r="J81" s="9" t="inlineStr"/>
-      <c r="K81" s="9" t="inlineStr"/>
+      <c r="K81" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/traktorist-по-полям-по-полям</t>
+        </is>
+      </c>
       <c r="L81" s="11" t="n">
         <v>0.002633333333333333</v>
       </c>
@@ -3980,7 +4244,11 @@
       <c r="H82" s="9" t="inlineStr"/>
       <c r="I82" s="10" t="inlineStr"/>
       <c r="J82" s="9" t="inlineStr"/>
-      <c r="K82" s="9" t="inlineStr"/>
+      <c r="K82" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/trupovoz</t>
+        </is>
+      </c>
       <c r="L82" s="11" t="n">
         <v>0.002747222222222223</v>
       </c>
@@ -4024,7 +4292,11 @@
       <c r="H83" s="9" t="inlineStr"/>
       <c r="I83" s="10" t="inlineStr"/>
       <c r="J83" s="9" t="inlineStr"/>
-      <c r="K83" s="9" t="inlineStr"/>
+      <c r="K83" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/valheim_-legacy-of-bronzebeard</t>
+        </is>
+      </c>
       <c r="L83" s="11" t="n">
         <v>0.003588310185185185</v>
       </c>
@@ -4064,7 +4336,11 @@
       <c r="H84" s="9" t="inlineStr"/>
       <c r="I84" s="10" t="inlineStr"/>
       <c r="J84" s="9" t="inlineStr"/>
-      <c r="K84" s="9" t="inlineStr"/>
+      <c r="K84" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/vea-мое-болото</t>
+        </is>
+      </c>
       <c r="L84" s="11" t="n">
         <v>0.001534953703703704</v>
       </c>
@@ -4104,7 +4380,11 @@
       <c r="H85" s="9" t="inlineStr"/>
       <c r="I85" s="10" t="inlineStr"/>
       <c r="J85" s="9" t="inlineStr"/>
-      <c r="K85" s="9" t="inlineStr"/>
+      <c r="K85" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/vomrakpadshiy-ballada-o-paladine-vo-mrake-v2</t>
+        </is>
+      </c>
       <c r="L85" s="11" t="n">
         <v>0.002031134259259259</v>
       </c>
@@ -4144,7 +4424,11 @@
       <c r="H86" s="9" t="inlineStr"/>
       <c r="I86" s="10" t="inlineStr"/>
       <c r="J86" s="9" t="inlineStr"/>
-      <c r="K86" s="9" t="inlineStr"/>
+      <c r="K86" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/warcrafter-вспоминаю-дни-когда-мир-был-жив</t>
+        </is>
+      </c>
       <c r="L86" s="11" t="n">
         <v>0.001331712962962963</v>
       </c>
@@ -4184,7 +4468,11 @@
       <c r="H87" s="9" t="inlineStr"/>
       <c r="I87" s="10" t="inlineStr"/>
       <c r="J87" s="9" t="inlineStr"/>
-      <c r="K87" s="9" t="inlineStr"/>
+      <c r="K87" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/warcrafter-вспоминаю-дни-v20</t>
+        </is>
+      </c>
       <c r="L87" s="11" t="n">
         <v>0.001362731481481481</v>
       </c>
@@ -4232,7 +4520,11 @@
       <c r="H88" s="9" t="inlineStr"/>
       <c r="I88" s="10" t="inlineStr"/>
       <c r="J88" s="9" t="inlineStr"/>
-      <c r="K88" s="9" t="inlineStr"/>
+      <c r="K88" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/wow-forever-тепло</t>
+        </is>
+      </c>
       <c r="L88" s="11" t="n">
         <v>0.002009722222222222</v>
       </c>
@@ -4280,7 +4572,11 @@
       <c r="H89" s="9" t="inlineStr"/>
       <c r="I89" s="10" t="inlineStr"/>
       <c r="J89" s="9" t="inlineStr"/>
-      <c r="K89" s="9" t="inlineStr"/>
+      <c r="K89" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/wow-forever</t>
+        </is>
+      </c>
       <c r="L89" s="11" t="n">
         <v>0.003616087962962963</v>
       </c>
@@ -4328,7 +4624,11 @@
       <c r="H90" s="9" t="inlineStr"/>
       <c r="I90" s="10" t="inlineStr"/>
       <c r="J90" s="9" t="inlineStr"/>
-      <c r="K90" s="9" t="inlineStr"/>
+      <c r="K90" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/а-может-просто-кисиком-стать</t>
+        </is>
+      </c>
       <c r="L90" s="11" t="n">
         <v>0.002907175925925926</v>
       </c>
@@ -4376,7 +4676,11 @@
       <c r="H91" s="9" t="inlineStr"/>
       <c r="I91" s="10" t="inlineStr"/>
       <c r="J91" s="9" t="inlineStr"/>
-      <c r="K91" s="9" t="inlineStr"/>
+      <c r="K91" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/аааа-бронзби́рд…-ну-шо-это-тако́е_</t>
+        </is>
+      </c>
       <c r="L91" s="11" t="n">
         <v>0.002066898148148148</v>
       </c>
@@ -4420,7 +4724,11 @@
       <c r="H92" s="9" t="inlineStr"/>
       <c r="I92" s="10" t="inlineStr"/>
       <c r="J92" s="9" t="inlineStr"/>
-      <c r="K92" s="9" t="inlineStr"/>
+      <c r="K92" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/аго́нит-в-шторме́</t>
+        </is>
+      </c>
       <c r="L92" s="11" t="n">
         <v>0.002223611111111111</v>
       </c>
@@ -4460,7 +4768,11 @@
       <c r="H93" s="9" t="inlineStr"/>
       <c r="I93" s="10" t="inlineStr"/>
       <c r="J93" s="9" t="inlineStr"/>
-      <c r="K93" s="9" t="inlineStr"/>
+      <c r="K93" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/агонит-эльфийские-руины</t>
+        </is>
+      </c>
       <c r="L93" s="11" t="n">
         <v>0.00318587962962963</v>
       </c>
@@ -4504,7 +4816,11 @@
       <c r="H94" s="9" t="inlineStr"/>
       <c r="I94" s="10" t="inlineStr"/>
       <c r="J94" s="9" t="inlineStr"/>
-      <c r="K94" s="9" t="inlineStr"/>
+      <c r="K94" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/айсберг-в-океане</t>
+        </is>
+      </c>
       <c r="L94" s="11" t="n">
         <v>0.003393865740740741</v>
       </c>
@@ -4552,7 +4868,11 @@
       <c r="H95" s="9" t="inlineStr"/>
       <c r="I95" s="10" t="inlineStr"/>
       <c r="J95" s="9" t="inlineStr"/>
-      <c r="K95" s="9" t="inlineStr"/>
+      <c r="K95" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/алмаз-из-говнистых-глубин</t>
+        </is>
+      </c>
       <c r="L95" s="11" t="n">
         <v>0.002481365740740741</v>
       </c>
@@ -4596,7 +4916,11 @@
       <c r="H96" s="9" t="inlineStr"/>
       <c r="I96" s="10" t="inlineStr"/>
       <c r="J96" s="9" t="inlineStr"/>
-      <c r="K96" s="9" t="inlineStr"/>
+      <c r="K96" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/альтушка-для-вия-homa-brut</t>
+        </is>
+      </c>
       <c r="L96" s="11" t="n">
         <v>0.002625</v>
       </c>
@@ -4640,7 +4964,11 @@
       <c r="H97" s="9" t="inlineStr"/>
       <c r="I97" s="10" t="inlineStr"/>
       <c r="J97" s="9" t="inlineStr"/>
-      <c r="K97" s="9" t="inlineStr"/>
+      <c r="K97" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/ассуми-самочка</t>
+        </is>
+      </c>
       <c r="L97" s="11" t="n">
         <v>0.000694675925925926</v>
       </c>
@@ -4684,7 +5012,11 @@
       <c r="H98" s="9" t="inlineStr"/>
       <c r="I98" s="10" t="inlineStr"/>
       <c r="J98" s="9" t="inlineStr"/>
-      <c r="K98" s="9" t="inlineStr"/>
+      <c r="K98" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/барон-ревиглаз-balenciaga</t>
+        </is>
+      </c>
       <c r="L98" s="11" t="n">
         <v>0.003703587962962963</v>
       </c>
@@ -4728,7 +5060,11 @@
       <c r="H99" s="9" t="inlineStr"/>
       <c r="I99" s="10" t="inlineStr"/>
       <c r="J99" s="9" t="inlineStr"/>
-      <c r="K99" s="9" t="inlineStr"/>
+      <c r="K99" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/барон-ревиглаз-пиратский-бенгер</t>
+        </is>
+      </c>
       <c r="L99" s="11" t="n">
         <v>0.002271064814814815</v>
       </c>
@@ -4772,7 +5108,11 @@
       <c r="H100" s="9" t="inlineStr"/>
       <c r="I100" s="10" t="inlineStr"/>
       <c r="J100" s="9" t="inlineStr"/>
-      <c r="K100" s="9" t="inlineStr"/>
+      <c r="K100" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/барон-ревиглаз-пиратский-косяк</t>
+        </is>
+      </c>
       <c r="L100" s="11" t="n">
         <v>0.002089120370370371</v>
       </c>
@@ -4820,7 +5160,11 @@
       <c r="H101" s="9" t="inlineStr"/>
       <c r="I101" s="10" t="inlineStr"/>
       <c r="J101" s="9" t="inlineStr"/>
-      <c r="K101" s="9" t="inlineStr"/>
+      <c r="K101" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/барон-ревиглаз-feat-dj-говнокрад-закрытие-бронзбирда</t>
+        </is>
+      </c>
       <c r="L101" s="11" t="n">
         <v>0.002136342592592593</v>
       </c>
@@ -4856,7 +5200,11 @@
       <c r="H102" s="9" t="inlineStr"/>
       <c r="I102" s="10" t="inlineStr"/>
       <c r="J102" s="9" t="inlineStr"/>
-      <c r="K102" s="9" t="inlineStr"/>
+      <c r="K102" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/бедство-элвиннского-леса</t>
+        </is>
+      </c>
       <c r="L102" s="11" t="n">
         <v>0.002345601851851852</v>
       </c>
@@ -4896,7 +5244,11 @@
       <c r="H103" s="9" t="inlineStr"/>
       <c r="I103" s="10" t="inlineStr"/>
       <c r="J103" s="9" t="inlineStr"/>
-      <c r="K103" s="9" t="inlineStr"/>
+      <c r="K103" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/блюз-эльфийские-руины</t>
+        </is>
+      </c>
       <c r="L103" s="11" t="n">
         <v>0.003268055555555556</v>
       </c>
@@ -4944,7 +5296,11 @@
       <c r="H104" s="9" t="inlineStr"/>
       <c r="I104" s="10" t="inlineStr"/>
       <c r="J104" s="9" t="inlineStr"/>
-      <c r="K104" s="9" t="inlineStr"/>
+      <c r="K104" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/бронзбирд-закрытие</t>
+        </is>
+      </c>
       <c r="L104" s="11" t="n">
         <v>0.002136342592592593</v>
       </c>
@@ -4988,7 +5344,11 @@
       <c r="H105" s="9" t="inlineStr"/>
       <c r="I105" s="10" t="inlineStr"/>
       <c r="J105" s="9" t="inlineStr"/>
-      <c r="K105" s="9" t="inlineStr"/>
+      <c r="K105" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/бухгалтер-гнилью</t>
+        </is>
+      </c>
       <c r="L105" s="11" t="n">
         <v>0.002198842592592593</v>
       </c>
@@ -5024,7 +5384,11 @@
       <c r="H106" s="9" t="inlineStr"/>
       <c r="I106" s="10" t="inlineStr"/>
       <c r="J106" s="9" t="inlineStr"/>
-      <c r="K106" s="9" t="inlineStr"/>
+      <c r="K106" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/в-склеп-древний-про́клятый-темный</t>
+        </is>
+      </c>
       <c r="L106" s="11" t="n">
         <v>0.002778356481481481</v>
       </c>
@@ -5100,7 +5464,11 @@
       <c r="H108" s="9" t="inlineStr"/>
       <c r="I108" s="10" t="inlineStr"/>
       <c r="J108" s="9" t="inlineStr"/>
-      <c r="K108" s="9" t="inlineStr"/>
+      <c r="K108" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/вперед-на-брбрбрбр</t>
+        </is>
+      </c>
       <c r="L108" s="11" t="n">
         <v>0.00276724537037037</v>
       </c>
@@ -5136,7 +5504,11 @@
       <c r="H109" s="9" t="inlineStr"/>
       <c r="I109" s="10" t="inlineStr"/>
       <c r="J109" s="9" t="inlineStr"/>
-      <c r="K109" s="9" t="inlineStr"/>
+      <c r="K109" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/гимн-чд-v3</t>
+        </is>
+      </c>
       <c r="L109" s="11" t="n">
         <v>0.002778356481481481</v>
       </c>
@@ -5172,7 +5544,11 @@
       <c r="H110" s="9" t="inlineStr"/>
       <c r="I110" s="10" t="inlineStr"/>
       <c r="J110" s="9" t="inlineStr"/>
-      <c r="K110" s="9" t="inlineStr"/>
+      <c r="K110" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/гимн-чд-но-это-аниме-jp</t>
+        </is>
+      </c>
       <c r="L110" s="11" t="n">
         <v>0.002778356481481481</v>
       </c>
@@ -5208,7 +5584,11 @@
       <c r="H111" s="9" t="inlineStr"/>
       <c r="I111" s="10" t="inlineStr"/>
       <c r="J111" s="9" t="inlineStr"/>
-      <c r="K111" s="9" t="inlineStr"/>
+      <c r="K111" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/гимн-чд-но-это-аниме-jp_metal</t>
+        </is>
+      </c>
       <c r="L111" s="11" t="n">
         <v>0.002550231481481481</v>
       </c>
@@ -5244,7 +5624,11 @@
       <c r="H112" s="9" t="inlineStr"/>
       <c r="I112" s="10" t="inlineStr"/>
       <c r="J112" s="9" t="inlineStr"/>
-      <c r="K112" s="9" t="inlineStr"/>
+      <c r="K112" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/гимн-чд</t>
+        </is>
+      </c>
       <c r="L112" s="11" t="n">
         <v>0.002778356481481481</v>
       </c>
@@ -5288,7 +5672,11 @@
       <c r="H113" s="9" t="inlineStr"/>
       <c r="I113" s="10" t="inlineStr"/>
       <c r="J113" s="9" t="inlineStr"/>
-      <c r="K113" s="9" t="inlineStr"/>
+      <c r="K113" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/грехопадение</t>
+        </is>
+      </c>
       <c r="L113" s="11" t="n">
         <v>0.003216898148148148</v>
       </c>
@@ -5332,7 +5720,11 @@
       <c r="H114" s="9" t="inlineStr"/>
       <c r="I114" s="10" t="inlineStr"/>
       <c r="J114" s="9" t="inlineStr"/>
-      <c r="K114" s="9" t="inlineStr"/>
+      <c r="K114" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/девять-кругов</t>
+        </is>
+      </c>
       <c r="L114" s="11" t="n">
         <v>0.0006736111111111112</v>
       </c>
@@ -5372,7 +5764,11 @@
       <c r="H115" s="9" t="inlineStr"/>
       <c r="I115" s="10" t="inlineStr"/>
       <c r="J115" s="9" t="inlineStr"/>
-      <c r="K115" s="9" t="inlineStr"/>
+      <c r="K115" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/дикий-прогрев</t>
+        </is>
+      </c>
       <c r="L115" s="11" t="n">
         <v>0.002041898148148148</v>
       </c>
@@ -5416,7 +5812,11 @@
       <c r="H116" s="9" t="inlineStr"/>
       <c r="I116" s="10" t="inlineStr"/>
       <c r="J116" s="9" t="inlineStr"/>
-      <c r="K116" s="9" t="inlineStr"/>
+      <c r="K116" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/димачка-вернулся-1топ</t>
+        </is>
+      </c>
       <c r="L116" s="11" t="n">
         <v>0.002604166666666667</v>
       </c>
@@ -5452,7 +5852,11 @@
       <c r="H117" s="9" t="inlineStr"/>
       <c r="I117" s="10" t="inlineStr"/>
       <c r="J117" s="9" t="inlineStr"/>
-      <c r="K117" s="9" t="inlineStr"/>
+      <c r="K117" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/др-денису</t>
+        </is>
+      </c>
       <c r="L117" s="11" t="n">
         <v>0.002172453703703704</v>
       </c>
@@ -7731,12 +8135,113 @@
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A3" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K130" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K16" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K17" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K18" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K19" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K20" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K21" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K22" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K23" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K24" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K25" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K26" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K27" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K28" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K29" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K30" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K31" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K32" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K33" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K34" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K35" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K36" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K37" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K38" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K39" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K40" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K41" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K42" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K43" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K44" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K45" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K46" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K47" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K48" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K49" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K50" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K51" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K52" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K53" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K54" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K55" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K56" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K57" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K58" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K59" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K60" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K61" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K62" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K63" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K64" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K65" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K66" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K67" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K68" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K69" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K70" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K71" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K72" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K73" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K74" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K75" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K76" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K77" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K78" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K79" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K80" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K81" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K82" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K83" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K84" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K85" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K86" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K87" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K88" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K89" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K90" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K91" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K92" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K93" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K94" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K95" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K96" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K97" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K98" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K99" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K100" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K101" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K102" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K103" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K104" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K105" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K106" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K108" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K109" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K110" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K111" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K112" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K113" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K114" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K115" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K116" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K117" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K130" r:id="rId103"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId104"/>
   </tableParts>
 </worksheet>
 </file>
@@ -8121,7 +8626,11 @@
       <c r="H12" s="9" t="inlineStr"/>
       <c r="I12" s="10" t="inlineStr"/>
       <c r="J12" s="9" t="inlineStr"/>
-      <c r="K12" s="9" t="inlineStr"/>
+      <c r="K12" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/cript-cover-den-1</t>
+        </is>
+      </c>
       <c r="L12" s="11" t="n">
         <v>0.002778356481481481</v>
       </c>
@@ -8157,7 +8666,11 @@
       <c r="H13" s="9" t="inlineStr"/>
       <c r="I13" s="10" t="inlineStr"/>
       <c r="J13" s="9" t="inlineStr"/>
-      <c r="K13" s="9" t="inlineStr"/>
+      <c r="K13" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/cryptonit-–-проклятие-крипты</t>
+        </is>
+      </c>
       <c r="L13" s="11" t="n">
         <v>0.002508101851851852</v>
       </c>
@@ -8193,7 +8706,11 @@
       <c r="H14" s="9" t="inlineStr"/>
       <c r="I14" s="10" t="inlineStr"/>
       <c r="J14" s="9" t="inlineStr"/>
-      <c r="K14" s="9" t="inlineStr"/>
+      <c r="K14" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/digital-fury</t>
+        </is>
+      </c>
       <c r="L14" s="11" t="n">
         <v>0.002633217592592592</v>
       </c>
@@ -8237,7 +8754,11 @@
       <c r="H15" s="9" t="inlineStr"/>
       <c r="I15" s="10" t="inlineStr"/>
       <c r="J15" s="9" t="inlineStr"/>
-      <c r="K15" s="9" t="inlineStr"/>
+      <c r="K15" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/dominus-agonetti-—-opera-sessions_-part-i-praeludium-in-ruinis-stratholmi-baro-tenebrosus</t>
+        </is>
+      </c>
       <c r="L15" s="11" t="n">
         <v>0.003261921296296296</v>
       </c>
@@ -8277,7 +8798,11 @@
       <c r="H16" s="9" t="inlineStr"/>
       <c r="I16" s="10" t="inlineStr"/>
       <c r="J16" s="9" t="inlineStr"/>
-      <c r="K16" s="9" t="inlineStr"/>
+      <c r="K16" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/edovuaruhaindo-fujōnaru-te-no-kayō</t>
+        </is>
+      </c>
       <c r="L16" s="11" t="n">
         <v>0.002778356481481481</v>
       </c>
@@ -8321,7 +8846,11 @@
       <c r="H17" s="9" t="inlineStr"/>
       <c r="I17" s="10" t="inlineStr"/>
       <c r="J17" s="9" t="inlineStr"/>
-      <c r="K17" s="9" t="inlineStr"/>
+      <c r="K17" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/fakmod-sirus</t>
+        </is>
+      </c>
       <c r="L17" s="11" t="n">
         <v>0.001800810185185185</v>
       </c>
@@ -8361,7 +8890,11 @@
       <c r="H18" s="9" t="inlineStr"/>
       <c r="I18" s="10" t="inlineStr"/>
       <c r="J18" s="9" t="inlineStr"/>
-      <c r="K18" s="9" t="inlineStr"/>
+      <c r="K18" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/fordring-о-король</t>
+        </is>
+      </c>
       <c r="L18" s="11" t="n">
         <v>0.001606134259259259</v>
       </c>
@@ -8405,7 +8938,11 @@
       <c r="H19" s="9" t="inlineStr"/>
       <c r="I19" s="10" t="inlineStr"/>
       <c r="J19" s="9" t="inlineStr"/>
-      <c r="K19" s="9" t="inlineStr"/>
+      <c r="K19" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/fuckmode-wow-sirus</t>
+        </is>
+      </c>
       <c r="L19" s="11" t="n">
         <v>0.001800578703703704</v>
       </c>
@@ -8449,7 +8986,11 @@
       <c r="H20" s="9" t="inlineStr"/>
       <c r="I20" s="10" t="inlineStr"/>
       <c r="J20" s="9" t="inlineStr"/>
-      <c r="K20" s="9" t="inlineStr"/>
+      <c r="K20" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/greywick-hill-мэрри-хоуп</t>
+        </is>
+      </c>
       <c r="L20" s="11" t="n">
         <v>0.00335150462962963</v>
       </c>
@@ -8489,7 +9030,11 @@
       <c r="H21" s="9" t="inlineStr"/>
       <c r="I21" s="10" t="inlineStr"/>
       <c r="J21" s="9" t="inlineStr"/>
-      <c r="K21" s="9" t="inlineStr"/>
+      <c r="K21" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/hastwood-ужас-в-вандермаре</t>
+        </is>
+      </c>
       <c r="L21" s="11" t="n">
         <v>0.002778356481481481</v>
       </c>
@@ -8525,7 +9070,11 @@
       <c r="H22" s="9" t="inlineStr"/>
       <c r="I22" s="10" t="inlineStr"/>
       <c r="J22" s="9" t="inlineStr"/>
-      <c r="K22" s="9" t="inlineStr"/>
+      <c r="K22" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/heilung_-_traust_skysoundcc</t>
+        </is>
+      </c>
       <c r="L22" s="11" t="n">
         <v>0.006855324074074074</v>
       </c>
@@ -8565,7 +9114,11 @@
       <c r="H23" s="9" t="inlineStr"/>
       <c r="I23" s="10" t="inlineStr"/>
       <c r="J23" s="9" t="inlineStr"/>
-      <c r="K23" s="9" t="inlineStr"/>
+      <c r="K23" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/hestia-discordiam-sugere</t>
+        </is>
+      </c>
       <c r="L23" s="11" t="n">
         <v>0.001683912037037037</v>
       </c>
@@ -8609,7 +9162,11 @@
       <c r="H24" s="9" t="inlineStr"/>
       <c r="I24" s="10" t="inlineStr"/>
       <c r="J24" s="9" t="inlineStr"/>
-      <c r="K24" s="9" t="inlineStr"/>
+      <c r="K24" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/homabrut-три-ночи</t>
+        </is>
+      </c>
       <c r="L24" s="11" t="n">
         <v>0.003156134259259259</v>
       </c>
@@ -8649,7 +9206,11 @@
       <c r="H25" s="9" t="inlineStr"/>
       <c r="I25" s="10" t="inlineStr"/>
       <c r="J25" s="9" t="inlineStr"/>
-      <c r="K25" s="9" t="inlineStr"/>
+      <c r="K25" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/kushnerit-cursed-crypt</t>
+        </is>
+      </c>
       <c r="L25" s="11" t="n">
         <v>0.002783564814814815</v>
       </c>
@@ -8689,7 +9250,11 @@
       <c r="H26" s="9" t="inlineStr"/>
       <c r="I26" s="10" t="inlineStr"/>
       <c r="J26" s="9" t="inlineStr"/>
-      <c r="K26" s="9" t="inlineStr"/>
+      <c r="K26" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/lightfair-мор-ладим</t>
+        </is>
+      </c>
       <c r="L26" s="11" t="n">
         <v>0.002145023148148149</v>
       </c>
@@ -8733,7 +9298,11 @@
       <c r="H27" s="9" t="inlineStr"/>
       <c r="I27" s="10" t="inlineStr"/>
       <c r="J27" s="9" t="inlineStr"/>
-      <c r="K27" s="9" t="inlineStr"/>
+      <c r="K27" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/morgenshtern-x-chd-саркофаг</t>
+        </is>
+      </c>
       <c r="L27" s="11" t="n">
         <v>0.002070023148148148</v>
       </c>
@@ -8773,7 +9342,11 @@
       <c r="H28" s="9" t="inlineStr"/>
       <c r="I28" s="10" t="inlineStr"/>
       <c r="J28" s="9" t="inlineStr"/>
-      <c r="K28" s="9" t="inlineStr"/>
+      <c r="K28" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/mrcrow-блю-юр</t>
+        </is>
+      </c>
       <c r="L28" s="11" t="n">
         <v>0.002141898148148148</v>
       </c>
@@ -8809,7 +9382,11 @@
       <c r="H29" s="9" t="inlineStr"/>
       <c r="I29" s="10" t="inlineStr"/>
       <c r="J29" s="9" t="inlineStr"/>
-      <c r="K29" s="9" t="inlineStr"/>
+      <c r="K29" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/neizvesten_-_podo_mnoj_penis_bolshoj_ochen_full_skysoundcc</t>
+        </is>
+      </c>
       <c r="L29" s="11" t="n">
         <v>0.001571064814814815</v>
       </c>
@@ -8849,7 +9426,11 @@
       <c r="H30" s="9" t="inlineStr"/>
       <c r="I30" s="10" t="inlineStr"/>
       <c r="J30" s="9" t="inlineStr"/>
-      <c r="K30" s="9" t="inlineStr"/>
+      <c r="K30" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/neoromant-о-король</t>
+        </is>
+      </c>
       <c r="L30" s="11" t="n">
         <v>0.001606134259259259</v>
       </c>
@@ -8889,7 +9470,11 @@
       <c r="H31" s="9" t="inlineStr"/>
       <c r="I31" s="10" t="inlineStr"/>
       <c r="J31" s="9" t="inlineStr"/>
-      <c r="K31" s="9" t="inlineStr"/>
+      <c r="K31" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/neuromant-agonito-no-kokoro</t>
+        </is>
+      </c>
       <c r="L31" s="11" t="n">
         <v>0.00226724537037037</v>
       </c>
@@ -8929,7 +9514,11 @@
       <c r="H32" s="9" t="inlineStr"/>
       <c r="I32" s="10" t="inlineStr"/>
       <c r="J32" s="9" t="inlineStr"/>
-      <c r="K32" s="9" t="inlineStr"/>
+      <c r="K32" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/neuromant-crypt</t>
+        </is>
+      </c>
       <c r="L32" s="11" t="n">
         <v>0.002778356481481481</v>
       </c>
@@ -8969,7 +9558,11 @@
       <c r="H33" s="9" t="inlineStr"/>
       <c r="I33" s="10" t="inlineStr"/>
       <c r="J33" s="9" t="inlineStr"/>
-      <c r="K33" s="9" t="inlineStr"/>
+      <c r="K33" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/neuromant-destiny</t>
+        </is>
+      </c>
       <c r="L33" s="11" t="n">
         <v>0.001761342592592593</v>
       </c>
@@ -9013,7 +9606,11 @@
       <c r="H34" s="9" t="inlineStr"/>
       <c r="I34" s="10" t="inlineStr"/>
       <c r="J34" s="9" t="inlineStr"/>
-      <c r="K34" s="9" t="inlineStr"/>
+      <c r="K34" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/neuromant-for-that-is-our-curse-arseny-kotofeev</t>
+        </is>
+      </c>
       <c r="L34" s="11" t="n">
         <v>0.002830324074074074</v>
       </c>
@@ -9053,7 +9650,11 @@
       <c r="H35" s="9" t="inlineStr"/>
       <c r="I35" s="10" t="inlineStr"/>
       <c r="J35" s="9" t="inlineStr"/>
-      <c r="K35" s="9" t="inlineStr"/>
+      <c r="K35" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/neuromant-mikurunomicon</t>
+        </is>
+      </c>
       <c r="L35" s="11" t="n">
         <v>0.001929398148148148</v>
       </c>
@@ -9097,7 +9698,11 @@
       <c r="H36" s="9" t="inlineStr"/>
       <c r="I36" s="10" t="inlineStr"/>
       <c r="J36" s="9" t="inlineStr"/>
-      <c r="K36" s="9" t="inlineStr"/>
+      <c r="K36" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/neuromant-singularity-1</t>
+        </is>
+      </c>
       <c r="L36" s="11" t="n">
         <v>0.002051157407407407</v>
       </c>
@@ -9137,7 +9742,11 @@
       <c r="H37" s="9" t="inlineStr"/>
       <c r="I37" s="10" t="inlineStr"/>
       <c r="J37" s="9" t="inlineStr"/>
-      <c r="K37" s="9" t="inlineStr"/>
+      <c r="K37" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/neuromant-артас-сын-мой-v-20</t>
+        </is>
+      </c>
       <c r="L37" s="11" t="n">
         <v>0.001666898148148148</v>
       </c>
@@ -9177,7 +9786,11 @@
       <c r="H38" s="9" t="inlineStr"/>
       <c r="I38" s="10" t="inlineStr"/>
       <c r="J38" s="9" t="inlineStr"/>
-      <c r="K38" s="9" t="inlineStr"/>
+      <c r="K38" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/neuromant-артас-сын-мой</t>
+        </is>
+      </c>
       <c r="L38" s="11" t="n">
         <v>0.001621990740740741</v>
       </c>
@@ -9217,7 +9830,11 @@
       <c r="H39" s="9" t="inlineStr"/>
       <c r="I39" s="10" t="inlineStr"/>
       <c r="J39" s="9" t="inlineStr"/>
-      <c r="K39" s="9" t="inlineStr"/>
+      <c r="K39" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/neuromant-баллада-об-андратосе</t>
+        </is>
+      </c>
       <c r="L39" s="11" t="n">
         <v>0.002778356481481481</v>
       </c>
@@ -9257,7 +9874,11 @@
       <c r="H40" s="9" t="inlineStr"/>
       <c r="I40" s="10" t="inlineStr"/>
       <c r="J40" s="9" t="inlineStr"/>
-      <c r="K40" s="9" t="inlineStr"/>
+      <c r="K40" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/neuromant-в-кругу-семьи-акт-iv</t>
+        </is>
+      </c>
       <c r="L40" s="11" t="n">
         <v>0.002709953703703704</v>
       </c>
@@ -9297,7 +9918,11 @@
       <c r="H41" s="9" t="inlineStr"/>
       <c r="I41" s="10" t="inlineStr"/>
       <c r="J41" s="9" t="inlineStr"/>
-      <c r="K41" s="9" t="inlineStr"/>
+      <c r="K41" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/neuromant-владыка-черной-длани-opening</t>
+        </is>
+      </c>
       <c r="L41" s="11" t="n">
         <v>0.002068634259259259</v>
       </c>
@@ -9337,7 +9962,11 @@
       <c r="H42" s="9" t="inlineStr"/>
       <c r="I42" s="10" t="inlineStr"/>
       <c r="J42" s="9" t="inlineStr"/>
-      <c r="K42" s="9" t="inlineStr"/>
+      <c r="K42" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/neuromant-воспоминание-о-лоретте</t>
+        </is>
+      </c>
       <c r="L42" s="11" t="n">
         <v>0.002171064814814815</v>
       </c>
@@ -9377,7 +10006,11 @@
       <c r="H43" s="9" t="inlineStr"/>
       <c r="I43" s="10" t="inlineStr"/>
       <c r="J43" s="9" t="inlineStr"/>
-      <c r="K43" s="9" t="inlineStr"/>
+      <c r="K43" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/neuromant-день-кузнечного-камня</t>
+        </is>
+      </c>
       <c r="L43" s="11" t="n">
         <v>0.001871990740740741</v>
       </c>
@@ -9417,7 +10050,11 @@
       <c r="H44" s="9" t="inlineStr"/>
       <c r="I44" s="10" t="inlineStr"/>
       <c r="J44" s="9" t="inlineStr"/>
-      <c r="K44" s="9" t="inlineStr"/>
+      <c r="K44" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/neuromant-дерьмадемон</t>
+        </is>
+      </c>
       <c r="L44" s="11" t="n">
         <v>0.002778356481481481</v>
       </c>
@@ -9457,7 +10094,11 @@
       <c r="H45" s="9" t="inlineStr"/>
       <c r="I45" s="10" t="inlineStr"/>
       <c r="J45" s="9" t="inlineStr"/>
-      <c r="K45" s="9" t="inlineStr"/>
+      <c r="K45" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/neuromant-клеть-nu-metal</t>
+        </is>
+      </c>
       <c r="L45" s="11" t="n">
         <v>0.001781134259259259</v>
       </c>
@@ -9497,7 +10138,11 @@
       <c r="H46" s="9" t="inlineStr"/>
       <c r="I46" s="10" t="inlineStr"/>
       <c r="J46" s="9" t="inlineStr"/>
-      <c r="K46" s="9" t="inlineStr"/>
+      <c r="K46" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/neuromant-клеть</t>
+        </is>
+      </c>
       <c r="L46" s="11" t="n">
         <v>0.002253935185185185</v>
       </c>
@@ -9537,7 +10182,11 @@
       <c r="H47" s="9" t="inlineStr"/>
       <c r="I47" s="10" t="inlineStr"/>
       <c r="J47" s="9" t="inlineStr"/>
-      <c r="K47" s="9" t="inlineStr"/>
+      <c r="K47" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/neuromant-край-бесконечно-истерзанный</t>
+        </is>
+      </c>
       <c r="L47" s="11" t="n">
         <v>0.001496412037037037</v>
       </c>
@@ -9577,7 +10226,11 @@
       <c r="H48" s="9" t="inlineStr"/>
       <c r="I48" s="10" t="inlineStr"/>
       <c r="J48" s="9" t="inlineStr"/>
-      <c r="K48" s="9" t="inlineStr"/>
+      <c r="K48" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/neuromant-миша-пошли-exclusive-lovesong-fm-radio-mix-r</t>
+        </is>
+      </c>
       <c r="L48" s="11" t="n">
         <v>0.001665046296296296</v>
       </c>
@@ -9617,7 +10270,11 @@
       <c r="H49" s="9" t="inlineStr"/>
       <c r="I49" s="10" t="inlineStr"/>
       <c r="J49" s="9" t="inlineStr"/>
-      <c r="K49" s="9" t="inlineStr"/>
+      <c r="K49" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/neuromant-ненависть</t>
+        </is>
+      </c>
       <c r="L49" s="11" t="n">
         <v>0.001736689814814815</v>
       </c>
@@ -9661,7 +10318,11 @@
       <c r="H50" s="9" t="inlineStr"/>
       <c r="I50" s="10" t="inlineStr"/>
       <c r="J50" s="9" t="inlineStr"/>
-      <c r="K50" s="9" t="inlineStr"/>
+      <c r="K50" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/neuromant-поднимите-веки-выше</t>
+        </is>
+      </c>
       <c r="L50" s="11" t="n">
         <v>0.002789699074074074</v>
       </c>
@@ -9701,7 +10362,11 @@
       <c r="H51" s="9" t="inlineStr"/>
       <c r="I51" s="10" t="inlineStr"/>
       <c r="J51" s="9" t="inlineStr"/>
-      <c r="K51" s="9" t="inlineStr"/>
+      <c r="K51" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/neuromant-полый</t>
+        </is>
+      </c>
       <c r="L51" s="11" t="n">
         <v>0.002554398148148148</v>
       </c>
@@ -9741,7 +10406,11 @@
       <c r="H52" s="9" t="inlineStr"/>
       <c r="I52" s="10" t="inlineStr"/>
       <c r="J52" s="9" t="inlineStr"/>
-      <c r="K52" s="9" t="inlineStr"/>
+      <c r="K52" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/neuromant-последний-полет-бабочки</t>
+        </is>
+      </c>
       <c r="L52" s="11" t="n">
         <v>0.001967824074074074</v>
       </c>
@@ -9781,7 +10450,11 @@
       <c r="H53" s="9" t="inlineStr"/>
       <c r="I53" s="10" t="inlineStr"/>
       <c r="J53" s="9" t="inlineStr"/>
-      <c r="K53" s="9" t="inlineStr"/>
+      <c r="K53" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/neuromant-проклятье-крипты-darkwave</t>
+        </is>
+      </c>
       <c r="L53" s="11" t="n">
         <v>0.002778356481481481</v>
       </c>
@@ -9821,7 +10494,11 @@
       <c r="H54" s="9" t="inlineStr"/>
       <c r="I54" s="10" t="inlineStr"/>
       <c r="J54" s="9" t="inlineStr"/>
-      <c r="K54" s="9" t="inlineStr"/>
+      <c r="K54" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/neuromant-проклятье-крипты</t>
+        </is>
+      </c>
       <c r="L54" s="11" t="n">
         <v>0.002783564814814815</v>
       </c>
@@ -9865,7 +10542,11 @@
       <c r="H55" s="9" t="inlineStr"/>
       <c r="I55" s="10" t="inlineStr"/>
       <c r="J55" s="9" t="inlineStr"/>
-      <c r="K55" s="9" t="inlineStr"/>
+      <c r="K55" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/neuromant-роксолана</t>
+        </is>
+      </c>
       <c r="L55" s="11" t="n">
         <v>0.002012268518518519</v>
       </c>
@@ -9905,7 +10586,11 @@
       <c r="H56" s="9" t="inlineStr"/>
       <c r="I56" s="10" t="inlineStr"/>
       <c r="J56" s="9" t="inlineStr"/>
-      <c r="K56" s="9" t="inlineStr"/>
+      <c r="K56" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/neuromant-слияние-вечности</t>
+        </is>
+      </c>
       <c r="L56" s="11" t="n">
         <v>0.001932523148148148</v>
       </c>
@@ -9945,7 +10630,11 @@
       <c r="H57" s="9" t="inlineStr"/>
       <c r="I57" s="10" t="inlineStr"/>
       <c r="J57" s="9" t="inlineStr"/>
-      <c r="K57" s="9" t="inlineStr"/>
+      <c r="K57" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/neuromant-терон</t>
+        </is>
+      </c>
       <c r="L57" s="11" t="n">
         <v>0.002457523148148148</v>
       </c>
@@ -9985,7 +10674,11 @@
       <c r="H58" s="9" t="inlineStr"/>
       <c r="I58" s="10" t="inlineStr"/>
       <c r="J58" s="9" t="inlineStr"/>
-      <c r="K58" s="9" t="inlineStr"/>
+      <c r="K58" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/neuromant-эйдолон-1</t>
+        </is>
+      </c>
       <c r="L58" s="11" t="n">
         <v>0.002783564814814815</v>
       </c>
@@ -10025,7 +10718,11 @@
       <c r="H59" s="9" t="inlineStr"/>
       <c r="I59" s="10" t="inlineStr"/>
       <c r="J59" s="9" t="inlineStr"/>
-      <c r="K59" s="9" t="inlineStr"/>
+      <c r="K59" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/neuromant-эйдолон-2</t>
+        </is>
+      </c>
       <c r="L59" s="11" t="n">
         <v>0.002783564814814815</v>
       </c>
@@ -10065,7 +10762,11 @@
       <c r="H60" s="9" t="inlineStr"/>
       <c r="I60" s="10" t="inlineStr"/>
       <c r="J60" s="9" t="inlineStr"/>
-      <c r="K60" s="9" t="inlineStr"/>
+      <c r="K60" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/neuromant-я-был-первым</t>
+        </is>
+      </c>
       <c r="L60" s="11" t="n">
         <v>0.002488657407407407</v>
       </c>
@@ -10105,7 +10806,11 @@
       <c r="H61" s="9" t="inlineStr"/>
       <c r="I61" s="10" t="inlineStr"/>
       <c r="J61" s="9" t="inlineStr"/>
-      <c r="K61" s="9" t="inlineStr"/>
+      <c r="K61" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/nuromanta-antipod-v-0666</t>
+        </is>
+      </c>
       <c r="L61" s="11" t="n">
         <v>0.002544212962962963</v>
       </c>
@@ -10141,7 +10846,11 @@
       <c r="H62" s="9" t="inlineStr"/>
       <c r="I62" s="10" t="inlineStr"/>
       <c r="J62" s="9" t="inlineStr"/>
-      <c r="K62" s="9" t="inlineStr"/>
+      <c r="K62" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/orchestra-de-la-poh-bain-russe</t>
+        </is>
+      </c>
       <c r="L62" s="11" t="n">
         <v>0.001703935185185185</v>
       </c>
@@ -10177,7 +10886,11 @@
       <c r="H63" s="9" t="inlineStr"/>
       <c r="I63" s="10" t="inlineStr"/>
       <c r="J63" s="9" t="inlineStr"/>
-      <c r="K63" s="9" t="inlineStr"/>
+      <c r="K63" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/powerwolf_ai_-_govnovoz_skysoundcc</t>
+        </is>
+      </c>
       <c r="L63" s="11" t="n">
         <v>0.002279398148148148</v>
       </c>
@@ -10213,7 +10926,11 @@
       <c r="H64" s="9" t="inlineStr"/>
       <c r="I64" s="10" t="inlineStr"/>
       <c r="J64" s="9" t="inlineStr"/>
-      <c r="K64" s="9" t="inlineStr"/>
+      <c r="K64" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/samhain-ball</t>
+        </is>
+      </c>
       <c r="L64" s="11" t="n">
         <v>0.001583564814814815</v>
       </c>
@@ -10257,7 +10974,11 @@
       <c r="H65" s="9" t="inlineStr"/>
       <c r="I65" s="10" t="inlineStr"/>
       <c r="J65" s="9" t="inlineStr"/>
-      <c r="K65" s="9" t="inlineStr"/>
+      <c r="K65" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/teron-я-был-первым-remastered</t>
+        </is>
+      </c>
       <c r="L65" s="11" t="n">
         <v>0.002138310185185185</v>
       </c>
@@ -10297,7 +11018,11 @@
       <c r="H66" s="9" t="inlineStr"/>
       <c r="I66" s="10" t="inlineStr"/>
       <c r="J66" s="9" t="inlineStr"/>
-      <c r="K66" s="9" t="inlineStr"/>
+      <c r="K66" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/trupovoz</t>
+        </is>
+      </c>
       <c r="L66" s="11" t="n">
         <v>0.002747222222222223</v>
       </c>
@@ -10337,7 +11062,11 @@
       <c r="H67" s="9" t="inlineStr"/>
       <c r="I67" s="10" t="inlineStr"/>
       <c r="J67" s="9" t="inlineStr"/>
-      <c r="K67" s="9" t="inlineStr"/>
+      <c r="K67" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/vea-мое-болото</t>
+        </is>
+      </c>
       <c r="L67" s="11" t="n">
         <v>0.001534953703703704</v>
       </c>
@@ -10377,7 +11106,11 @@
       <c r="H68" s="9" t="inlineStr"/>
       <c r="I68" s="10" t="inlineStr"/>
       <c r="J68" s="9" t="inlineStr"/>
-      <c r="K68" s="9" t="inlineStr"/>
+      <c r="K68" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/vomrakpadshiy-ballada-o-paladine-vo-mrake-v2</t>
+        </is>
+      </c>
       <c r="L68" s="11" t="n">
         <v>0.002031134259259259</v>
       </c>
@@ -10417,7 +11150,11 @@
       <c r="H69" s="9" t="inlineStr"/>
       <c r="I69" s="10" t="inlineStr"/>
       <c r="J69" s="9" t="inlineStr"/>
-      <c r="K69" s="9" t="inlineStr"/>
+      <c r="K69" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/warcrafter-вспоминаю-дни-когда-мир-был-жив</t>
+        </is>
+      </c>
       <c r="L69" s="11" t="n">
         <v>0.001331712962962963</v>
       </c>
@@ -10457,7 +11194,11 @@
       <c r="H70" s="9" t="inlineStr"/>
       <c r="I70" s="10" t="inlineStr"/>
       <c r="J70" s="9" t="inlineStr"/>
-      <c r="K70" s="9" t="inlineStr"/>
+      <c r="K70" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/warcrafter-вспоминаю-дни-v20</t>
+        </is>
+      </c>
       <c r="L70" s="11" t="n">
         <v>0.001362731481481481</v>
       </c>
@@ -10501,7 +11242,11 @@
       <c r="H71" s="9" t="inlineStr"/>
       <c r="I71" s="10" t="inlineStr"/>
       <c r="J71" s="9" t="inlineStr"/>
-      <c r="K71" s="9" t="inlineStr"/>
+      <c r="K71" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/альтушка-для-вия-homa-brut</t>
+        </is>
+      </c>
       <c r="L71" s="11" t="n">
         <v>0.002625</v>
       </c>
@@ -10537,7 +11282,11 @@
       <c r="H72" s="9" t="inlineStr"/>
       <c r="I72" s="10" t="inlineStr"/>
       <c r="J72" s="9" t="inlineStr"/>
-      <c r="K72" s="9" t="inlineStr"/>
+      <c r="K72" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/бедство-элвиннского-леса</t>
+        </is>
+      </c>
       <c r="L72" s="11" t="n">
         <v>0.002345601851851852</v>
       </c>
@@ -10573,7 +11322,11 @@
       <c r="H73" s="9" t="inlineStr"/>
       <c r="I73" s="10" t="inlineStr"/>
       <c r="J73" s="9" t="inlineStr"/>
-      <c r="K73" s="9" t="inlineStr"/>
+      <c r="K73" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/в-склеп-древний-про́клятый-темный</t>
+        </is>
+      </c>
       <c r="L73" s="11" t="n">
         <v>0.002778356481481481</v>
       </c>
@@ -10649,7 +11402,11 @@
       <c r="H75" s="9" t="inlineStr"/>
       <c r="I75" s="10" t="inlineStr"/>
       <c r="J75" s="9" t="inlineStr"/>
-      <c r="K75" s="9" t="inlineStr"/>
+      <c r="K75" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/вперед-на-брбрбрбр</t>
+        </is>
+      </c>
       <c r="L75" s="11" t="n">
         <v>0.00276724537037037</v>
       </c>
@@ -10685,7 +11442,11 @@
       <c r="H76" s="9" t="inlineStr"/>
       <c r="I76" s="10" t="inlineStr"/>
       <c r="J76" s="9" t="inlineStr"/>
-      <c r="K76" s="9" t="inlineStr"/>
+      <c r="K76" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/гимн-чд-v3</t>
+        </is>
+      </c>
       <c r="L76" s="11" t="n">
         <v>0.002778356481481481</v>
       </c>
@@ -10721,7 +11482,11 @@
       <c r="H77" s="9" t="inlineStr"/>
       <c r="I77" s="10" t="inlineStr"/>
       <c r="J77" s="9" t="inlineStr"/>
-      <c r="K77" s="9" t="inlineStr"/>
+      <c r="K77" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/гимн-чд-но-это-аниме-jp</t>
+        </is>
+      </c>
       <c r="L77" s="11" t="n">
         <v>0.002778356481481481</v>
       </c>
@@ -10757,7 +11522,11 @@
       <c r="H78" s="9" t="inlineStr"/>
       <c r="I78" s="10" t="inlineStr"/>
       <c r="J78" s="9" t="inlineStr"/>
-      <c r="K78" s="9" t="inlineStr"/>
+      <c r="K78" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/гимн-чд-но-это-аниме-jp_metal</t>
+        </is>
+      </c>
       <c r="L78" s="11" t="n">
         <v>0.002550231481481481</v>
       </c>
@@ -10793,7 +11562,11 @@
       <c r="H79" s="9" t="inlineStr"/>
       <c r="I79" s="10" t="inlineStr"/>
       <c r="J79" s="9" t="inlineStr"/>
-      <c r="K79" s="9" t="inlineStr"/>
+      <c r="K79" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/гимн-чд</t>
+        </is>
+      </c>
       <c r="L79" s="11" t="n">
         <v>0.002778356481481481</v>
       </c>
@@ -10829,7 +11602,11 @@
       <c r="H80" s="9" t="inlineStr"/>
       <c r="I80" s="10" t="inlineStr"/>
       <c r="J80" s="9" t="inlineStr"/>
-      <c r="K80" s="9" t="inlineStr"/>
+      <c r="K80" s="13" t="inlineStr">
+        <is>
+          <t>https://audius.co/Durachok/др-денису</t>
+        </is>
+      </c>
       <c r="L80" s="11" t="n">
         <v>0.002172453703703704</v>
       </c>
@@ -11532,11 +12309,79 @@
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A3" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K12" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K13" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K14" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K15" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K16" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K17" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K18" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K19" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K20" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K21" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K22" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K23" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K24" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K25" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K26" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K27" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K28" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K29" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K30" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K31" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K32" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K33" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K34" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K35" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K36" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K37" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K38" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K39" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K40" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K41" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K42" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K43" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K44" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K45" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K46" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K47" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K48" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K49" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K50" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K51" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K52" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K53" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K54" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K55" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K56" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K57" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K58" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K59" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K60" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K61" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K62" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K63" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K64" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K65" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K66" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K67" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K68" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K69" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K70" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K71" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K72" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K73" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K75" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K76" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K77" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K78" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K79" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K80" r:id="rId69"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId70"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>